<commit_message>
update: add VLM model
</commit_message>
<xml_diff>
--- a/composeApp/model/model.xlsx
+++ b/composeApp/model/model.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="44">
   <si>
     <t>model</t>
   </si>
@@ -28,6 +28,12 @@
     <t>enable_thinking</t>
   </si>
   <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>disabled</t>
+  </si>
+  <si>
     <t>desc</t>
   </si>
   <si>
@@ -37,10 +43,13 @@
     <t>Qwen3</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="11"/>
+    <t>LLM</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">Qwen3-8B </t>
@@ -48,7 +57,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是通义千问系列的最新大语言模型，拥有</t>
@@ -56,7 +65,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 8.2B </t>
@@ -64,7 +73,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>参数量。该模型独特地支持在思考模式（适用于复杂逻辑推理、数学和编程）和非思考模式（适用于高效的通用对话）之间无缝切换，显著增强了推理能力。模型在数学、代码生成和常识逻辑推理上表现优异，并在创意写作、角色扮演和多轮对话等方面展现出卓越的人类偏好对齐能力。此外，该模型支持</t>
@@ -72,7 +81,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 100 </t>
@@ -80,7 +89,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>多种语言和方言，具备出色的多语言指令遵循和翻译能力</t>
@@ -96,7 +105,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">DeepSeek-R1-Distill-Qwen-7B </t>
@@ -104,7 +113,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是基于</t>
@@ -112,7 +121,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> Qwen2.5-Math-7B </t>
@@ -120,7 +129,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>通过知识蒸馏得到的模型。该模型使用</t>
@@ -128,7 +137,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> DeepSeek-R1 </t>
@@ -136,7 +145,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>生成的</t>
@@ -144,7 +153,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 80 </t>
@@ -152,7 +161,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>万个精选样本进行微调，展现出优秀的推理能力。在多个基准测试中表现出色，其中在</t>
@@ -160,7 +169,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> MATH-500 </t>
@@ -168,7 +177,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>上达到了</t>
@@ -176,7 +185,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 92.8% </t>
@@ -184,7 +193,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>的准确率，在</t>
@@ -192,7 +201,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> AIME 2024 </t>
@@ -200,7 +209,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>上达到了</t>
@@ -208,7 +217,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 55.5% </t>
@@ -216,7 +225,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>的通过率，在</t>
@@ -224,7 +233,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> CodeForces </t>
@@ -232,7 +241,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>上获得了</t>
@@ -240,7 +249,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 1189 </t>
@@ -248,7 +257,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>的评分，作为</t>
@@ -256,7 +265,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 7B </t>
@@ -264,7 +273,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>规模的模型展示了较强的数学和编程能力</t>
@@ -277,7 +286,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">DeepSeek-R1-Distill-Qwen-1.5B </t>
@@ -285,7 +294,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是基于</t>
@@ -293,7 +302,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> Qwen2.5-Math-1.5B </t>
@@ -301,7 +310,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>通过知识蒸馏得到的模型。该模型使用</t>
@@ -309,7 +318,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> DeepSeek-R1 </t>
@@ -317,7 +326,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>生成的</t>
@@ -325,7 +334,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 80 </t>
@@ -333,7 +342,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>万个精选样本进行微调，在多个基准测试中展现出不错的性能。作为一个轻量级模型，在</t>
@@ -341,7 +350,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> MATH-500 </t>
@@ -349,7 +358,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>上达到了</t>
@@ -357,7 +366,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 83.9% </t>
@@ -365,7 +374,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>的准确率，在</t>
@@ -373,7 +382,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> AIME 2024 </t>
@@ -381,7 +390,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>上达到了</t>
@@ -389,7 +398,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 28.9% </t>
@@ -397,7 +406,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>的通过率，在</t>
@@ -405,7 +414,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> CodeForces </t>
@@ -413,7 +422,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>上获得了</t>
@@ -421,7 +430,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 954 </t>
@@ -429,7 +438,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>的评分，显示出超出其参数规模的推理能力</t>
@@ -445,7 +454,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">Qwen2.5-7B-Instruct </t>
@@ -453,7 +462,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是阿里云发布的最新大语言模型系列之一。该</t>
@@ -461,7 +470,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 7B </t>
@@ -469,7 +478,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>模型在编码和数学等领域具有显著改进的能力。该模型还提供了多语言支持，覆盖超过</t>
@@ -477,7 +486,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 29 </t>
@@ -485,7 +494,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>种语言，包括中文、英文等。模型在指令跟随、理解结构化数据以及生成结构化输出（尤其是</t>
@@ -493,7 +502,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> JSON</t>
@@ -501,7 +510,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>）方面都有显著提升</t>
@@ -514,7 +523,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">Qwen2.5-Coder-7B-Instruct </t>
@@ -522,7 +531,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是阿里云发布的代码特定大语言模型系列的最新版本。该模型在</t>
@@ -530,7 +539,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> Qwen2.5 </t>
@@ -538,7 +547,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>的基础上，通过</t>
@@ -546,7 +555,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 5.5 </t>
@@ -554,7 +563,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>万亿个</t>
@@ -562,7 +571,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> tokens </t>
@@ -570,7 +579,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>的训练，显著提升了代码生成、推理和修复能力。它不仅增强了编码能力，还保持了数学和通用能力的优势。模型为代码智能体等实际应用提供了更全面的基础</t>
@@ -578,7 +587,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t>"</t>
@@ -591,7 +600,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t>书生</t>
@@ -599,7 +608,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'JetBrains Mono'"/>
       </rPr>
       <t>·</t>
@@ -607,7 +616,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t>浦语</t>
@@ -617,7 +626,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">InternLM2.5-7B-Chat </t>
@@ -625,7 +634,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是一个开源的对话模型，基于</t>
@@ -633,7 +642,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> InternLM2 </t>
@@ -641,7 +650,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>架构开发。该</t>
@@ -649,7 +658,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 7B </t>
@@ -657,7 +666,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>参数规模的模型专注于对话生成任务，支持中英双语交互。模型采用了最新的训练技术，旨在提供流畅、智能的对话体验。</t>
@@ -665,7 +674,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">InternLM2.5-7B-Chat </t>
@@ -673,7 +682,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>适用于各种对话应用场景，包括但不限于智能客服、个人助手等领域</t>
@@ -689,7 +698,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">Qwen2-7B-Instruct </t>
@@ -697,7 +706,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是</t>
@@ -705,7 +714,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> Qwen2 </t>
@@ -713,7 +722,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>系列中的指令微调大语言模型，参数规模为</t>
@@ -721,7 +730,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 7B</t>
@@ -729,7 +738,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>。该模型基于</t>
@@ -737,7 +746,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> Transformer </t>
@@ -745,7 +754,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>架构，采用了</t>
@@ -753,7 +762,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> SwiGLU </t>
@@ -761,7 +770,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>激活函数、注意力</t>
@@ -769,7 +778,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> QKV </t>
@@ -777,7 +786,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>偏置和组查询注意力等技术。它能够处理大规模输入。该模型在语言理解、生成、多语言能力、编码、数学和推理等多个基准测试中表现出色，超越了大多数开源模型，并在某些任务上展现出与专有模型相当的竞争力。</t>
@@ -785,7 +794,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">Qwen2-7B-Instruct </t>
@@ -793,7 +802,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>在多项评测中均优于</t>
@@ -801,7 +810,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> Qwen1.5-7B-Chat</t>
@@ -809,7 +818,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>，显示出显著的性能提升</t>
@@ -822,7 +831,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">Qwen2-1.5B-Instruct </t>
@@ -830,7 +839,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是</t>
@@ -838,7 +847,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> Qwen2 </t>
@@ -846,7 +855,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>系列中的指令微调大语言模型，参数规模为</t>
@@ -854,7 +863,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 1.5B</t>
@@ -862,7 +871,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>。该模型基于</t>
@@ -870,7 +879,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> Transformer </t>
@@ -878,7 +887,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>架构，采用了</t>
@@ -886,7 +895,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> SwiGLU </t>
@@ -894,7 +903,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>激活函数、注意力</t>
@@ -902,7 +911,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> QKV </t>
@@ -910,7 +919,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>偏置和组查询注意力等技术。它在语言理解、生成、多语言能力、编码、数学和推理等多个基准测试中表现出色，超越了大多数开源模型。与</t>
@@ -918,7 +927,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> Qwen1.5-1.8B-Chat </t>
@@ -926,7 +935,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>相比，</t>
@@ -934,7 +943,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">Qwen2-1.5B-Instruct </t>
@@ -942,7 +951,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>在</t>
@@ -950,7 +959,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> MMLU</t>
@@ -958,7 +967,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>、</t>
@@ -966,7 +975,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t>HumanEval</t>
@@ -974,7 +983,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>、</t>
@@ -982,7 +991,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t>GSM8K</t>
@@ -990,7 +999,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>、</t>
@@ -998,7 +1007,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">C-Eval </t>
@@ -1006,7 +1015,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>和</t>
@@ -1014,7 +1023,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> IFEval </t>
@@ -1022,7 +1031,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>等测试中均显示出显著的性能提升，尽管参数量略少</t>
@@ -1035,7 +1044,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t>智谱</t>
@@ -1043,7 +1052,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'JetBrains Mono'"/>
       </rPr>
       <t>AI</t>
@@ -1053,7 +1062,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">GLM-Z1-9B-0414 </t>
@@ -1061,7 +1070,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是</t>
@@ -1069,7 +1078,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> GLM </t>
@@ -1077,7 +1086,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>系列的小型模型，仅有</t>
@@ -1085,7 +1094,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 90 </t>
@@ -1093,7 +1102,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>亿参数，但保持了开源传统的同时展现出惊人的能力。尽管规模较小，该模型在数学推理和通用任务上仍表现出色，其总体性能在同等规模的开源模型中已处于领先水平。研究团队采用了与大模型相同的一系列技术进行训练，使其在资源受限的场景中能够实现效率与效果的绝佳平衡，为寻求轻量级部署的用户提供强大选择。特别是在资源受限的场景下，该模型可以很好地在效率与效果之间取得平衡，为需要轻量化部署的用户提供强有力的选择</t>
@@ -1106,7 +1115,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">GLM-4-9B-0414 </t>
@@ -1114,7 +1123,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是</t>
@@ -1122,7 +1131,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> GLM </t>
@@ -1130,7 +1139,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>系列的小型模型，拥有</t>
@@ -1138,7 +1147,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 90 </t>
@@ -1146,7 +1155,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>亿参数。该模型继承了</t>
@@ -1154,7 +1163,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> GLM-4-32B </t>
@@ -1162,7 +1171,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>系列的技术特点，但提供了更轻量级的部署选择。尽管规模较小，</t>
@@ -1170,7 +1179,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">GLM-4-9B-0414 </t>
@@ -1178,7 +1187,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>仍在代码生成、网页设计、</t>
@@ -1186,7 +1195,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">SVG </t>
@@ -1194,7 +1203,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>图形生成和基于搜索的写作等任务上展现出色能力。该模型还支持函数调用功能，可以调用外部工具以扩展其能力范围。模型在资源受限的场景中表现出良好的效率与效果平衡，为需要在计算资源有限条件下部署</t>
@@ -1202,7 +1211,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> AI </t>
@@ -1210,7 +1219,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>模型的用户提供了强大选择。与其他同系列模型一样，</t>
@@ -1218,7 +1227,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">GLM-4-9B-0414 </t>
@@ -1226,7 +1235,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>也展示了在各种基准测试中的竞争性能力</t>
@@ -1239,7 +1248,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">GLM-4-9B-Chat </t>
@@ -1247,7 +1256,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是智谱</t>
@@ -1255,7 +1264,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> AI </t>
@@ -1263,7 +1272,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>推出的</t>
@@ -1271,7 +1280,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> GLM-4 </t>
@@ -1279,7 +1288,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>系列预训练模型中的开源版本。该模型在语义、数学、推理、代码和知识等多个方面表现出色。除了支持多轮对话外，</t>
@@ -1287,7 +1296,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">GLM-4-9B-Chat </t>
@@ -1295,7 +1304,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>还具备网页浏览、代码执行、自定义工具调用（</t>
@@ -1303,7 +1312,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t>Function Call</t>
@@ -1311,7 +1320,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>）和长文本推理等高级功能。模型支持</t>
@@ -1319,7 +1328,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 26 </t>
@@ -1327,7 +1336,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>种语言，包括中文、英文、日语、韩语和德语等。在多项基准测试中，</t>
@@ -1335,7 +1344,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">GLM-4-9B-Chat </t>
@@ -1343,7 +1352,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>展现了优秀的性能，如</t>
@@ -1351,7 +1360,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> AlignBench-v2</t>
@@ -1359,7 +1368,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>、</t>
@@ -1367,7 +1376,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t>MT-Bench</t>
@@ -1375,7 +1384,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>、</t>
@@ -1383,7 +1392,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">MMLU </t>
@@ -1391,7 +1400,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>和</t>
@@ -1399,7 +1408,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> C-Eval </t>
@@ -1407,7 +1416,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>等。该模型支持最大</t>
@@ -1415,7 +1424,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 128K </t>
@@ -1423,7 +1432,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>的上下文长度，适用于学术研究和商业应用</t>
@@ -1436,7 +1445,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">ChatGLM3-6B </t>
@@ -1444,7 +1453,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>是</t>
@@ -1452,7 +1461,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> ChatGLM </t>
@@ -1460,7 +1469,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>系列的开源模型，由智谱</t>
@@ -1468,7 +1477,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> AI </t>
@@ -1476,7 +1485,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>开发。该模型保留了前代模型的优秀特性，如对话流畅和部署门槛低，同时引入了新的特性。它采用了更多样的训练数据、更充分的训练步数和更合理的训练策略，在</t>
@@ -1484,7 +1493,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> 10B </t>
@@ -1492,7 +1501,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>以下的预训练模型中表现出色。</t>
@@ -1500,7 +1509,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve">ChatGLM3-6B </t>
@@ -1508,7 +1517,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>支持多轮对话、工具调用、代码执行和</t>
@@ -1516,7 +1525,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> Agent </t>
@@ -1524,7 +1533,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>任务等复杂场景。除对话模型外，还开源了基础模型</t>
@@ -1532,7 +1541,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> ChatGLM-6B-Base </t>
@@ -1540,7 +1549,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>和长文本对话模型</t>
@@ -1548,7 +1557,7 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="Verdana"/>
       </rPr>
       <t xml:space="preserve"> ChatGLM3-6B-32K</t>
@@ -1556,11 +1565,26 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="'Menlo-Regular'"/>
       </rPr>
       <t>。该模型对学术研究完全开放，在登记后也允许免费商业使用</t>
     </r>
+  </si>
+  <si>
+    <t>deepseek-ai/DeepSeek-R1-0528-Qwen3-8B</t>
+  </si>
+  <si>
+    <t>DeepSeek-R1-0528-Qwen3-8B 是通过从 DeepSeek-R1-0528 模型蒸馏思维链到 Qwen3 8B Base 获得的模型。该模型在开源模型中达到了最先进（SOTA）的性能，在 AIME 2024 测试中超越了 Qwen3 8B 10%，并达到了 Qwen3-235B-thinking 的性能水平。该模型在数学推理、编程和通用逻辑等多个基准测试中表现出色，其架构与 Qwen3-8B 相同，但共享 DeepSeek-R1-0528 的分词器配置</t>
+  </si>
+  <si>
+    <t>THUDM/GLM-4.1V-9B-Thinking</t>
+  </si>
+  <si>
+    <t>VLM</t>
+  </si>
+  <si>
+    <t>GLM-4.1V-9B-Thinking 是由智谱 AI 和清华大学 KEG 实验室联合发布的一款开源视觉语言模型（VLM），专为处理复杂的多模态认知任务而设计。该模型基于 GLM-4-9B-0414 基础模型，通过引入“思维链”（Chain-of-Thought）推理机制和采用强化学习策略，显著提升了其跨模态的推理能力和稳定性。作为一个 9B 参数规模的轻量级模型，它在部署效率和性能之间取得了平衡，在 28 项权威评测基准中，有 18 项的表现持平甚至超越了 72B 参数规模的 Qwen-2.5-VL-72B。该模型不仅在图文理解、数学科学推理、视频理解等任务上表现卓越，还支持高达 4K 分辨率的图像和任意宽高比输入</t>
   </si>
 </sst>
 </file>
@@ -1593,11 +1617,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color indexed="11"/>
-      <name val="等线"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color indexed="12"/>
       <name val="等线"/>
     </font>
@@ -1608,17 +1627,22 @@
     </font>
     <font>
       <sz val="10"/>
-      <color indexed="11"/>
+      <color indexed="14"/>
+      <name val="等线"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="12"/>
       <name val="Verdana"/>
     </font>
     <font>
       <sz val="10"/>
-      <color indexed="11"/>
+      <color indexed="12"/>
       <name val="'Menlo-Regular'"/>
     </font>
     <font>
       <sz val="10"/>
-      <color indexed="11"/>
+      <color indexed="12"/>
       <name val="'JetBrains Mono'"/>
     </font>
   </fonts>
@@ -1631,7 +1655,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="14"/>
+        <fgColor indexed="10"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -1646,16 +1670,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="10"/>
+        <color indexed="11"/>
       </left>
       <right style="thin">
-        <color indexed="10"/>
+        <color indexed="11"/>
       </right>
       <top style="thin">
-        <color indexed="10"/>
+        <color indexed="11"/>
       </top>
       <bottom style="thin">
-        <color indexed="10"/>
+        <color indexed="11"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1665,32 +1689,38 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1711,11 +1741,11 @@
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
       <rgbColor rgb="ffc77dbb"/>
+      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffaaaaaa"/>
       <rgbColor rgb="ff6aab73"/>
       <rgbColor rgb="ff2aacb8"/>
       <rgbColor rgb="ffcf8e6d"/>
-      <rgbColor rgb="ffffffff"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1914,12 +1944,12 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="19050" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1951,10 +1981,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -2193,12 +2223,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="19050" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -2502,10 +2532,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -2750,14 +2780,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultColWidth="14" defaultRowHeight="18" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="38.4219" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.8125" style="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="6" width="14" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="14" style="1" customWidth="1"/>
+    <col min="4" max="8" width="14" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="14" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2779,13 +2809,19 @@
       <c r="F1" t="s" s="2">
         <v>5</v>
       </c>
+      <c r="G1" t="s" s="2">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s" s="2">
+        <v>7</v>
+      </c>
     </row>
     <row r="2" ht="17" customHeight="1">
       <c r="A2" t="s" s="3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s" s="3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C2" s="4">
         <v>0</v>
@@ -2797,15 +2833,19 @@
         <v>1</v>
       </c>
       <c r="F2" t="s" s="7">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="G2" s="8"/>
+      <c r="H2" t="s" s="9">
+        <v>11</v>
       </c>
     </row>
     <row r="3" ht="17" customHeight="1">
       <c r="A3" t="s" s="3">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s" s="3">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C3" s="4">
         <v>0</v>
@@ -2813,17 +2853,21 @@
       <c r="D3" s="5">
         <v>16384</v>
       </c>
-      <c r="E3" s="8"/>
+      <c r="E3" s="10"/>
       <c r="F3" t="s" s="7">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="G3" s="10"/>
+      <c r="H3" t="s" s="9">
+        <v>14</v>
       </c>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" t="s" s="3">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s" s="3">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C4" s="4">
         <v>0</v>
@@ -2831,17 +2875,23 @@
       <c r="D4" s="5">
         <v>16384</v>
       </c>
-      <c r="E4" s="8"/>
+      <c r="E4" s="10"/>
       <c r="F4" t="s" s="7">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="G4" t="b" s="6">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s" s="9">
+        <v>16</v>
       </c>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" t="s" s="3">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s" s="3">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C5" s="4">
         <v>0</v>
@@ -2849,17 +2899,21 @@
       <c r="D5" s="5">
         <v>4096</v>
       </c>
-      <c r="E5" s="8"/>
+      <c r="E5" s="10"/>
       <c r="F5" t="s" s="7">
-        <v>16</v>
+        <v>10</v>
+      </c>
+      <c r="G5" s="10"/>
+      <c r="H5" t="s" s="9">
+        <v>19</v>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" t="s" s="3">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s" s="3">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C6" s="4">
         <v>0</v>
@@ -2867,17 +2921,21 @@
       <c r="D6" s="5">
         <v>4096</v>
       </c>
-      <c r="E6" s="8"/>
+      <c r="E6" s="10"/>
       <c r="F6" t="s" s="7">
-        <v>18</v>
+        <v>10</v>
+      </c>
+      <c r="G6" s="10"/>
+      <c r="H6" t="s" s="9">
+        <v>21</v>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" t="s" s="3">
-        <v>19</v>
-      </c>
-      <c r="B7" t="s" s="7">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="B7" t="s" s="9">
+        <v>23</v>
       </c>
       <c r="C7" s="4">
         <v>0</v>
@@ -2885,17 +2943,21 @@
       <c r="D7" s="5">
         <v>4096</v>
       </c>
-      <c r="E7" s="8"/>
+      <c r="E7" s="10"/>
       <c r="F7" t="s" s="7">
-        <v>21</v>
+        <v>10</v>
+      </c>
+      <c r="G7" s="10"/>
+      <c r="H7" t="s" s="9">
+        <v>24</v>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" t="s" s="3">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s" s="3">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C8" s="4">
         <v>0</v>
@@ -2903,17 +2965,21 @@
       <c r="D8" s="5">
         <v>4096</v>
       </c>
-      <c r="E8" s="8"/>
+      <c r="E8" s="10"/>
       <c r="F8" t="s" s="7">
-        <v>24</v>
+        <v>10</v>
+      </c>
+      <c r="G8" s="10"/>
+      <c r="H8" t="s" s="9">
+        <v>27</v>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" t="s" s="3">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s" s="3">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C9" s="4">
         <v>0</v>
@@ -2921,17 +2987,23 @@
       <c r="D9" s="5">
         <v>4096</v>
       </c>
-      <c r="E9" s="8"/>
+      <c r="E9" s="10"/>
       <c r="F9" t="s" s="7">
-        <v>26</v>
+        <v>10</v>
+      </c>
+      <c r="G9" t="b" s="6">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s" s="9">
+        <v>29</v>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="B10" t="s" s="7">
-        <v>28</v>
+        <v>30</v>
+      </c>
+      <c r="B10" t="s" s="9">
+        <v>31</v>
       </c>
       <c r="C10" s="4">
         <v>0</v>
@@ -2939,17 +3011,21 @@
       <c r="D10" s="5">
         <v>8192</v>
       </c>
-      <c r="E10" s="8"/>
+      <c r="E10" s="10"/>
       <c r="F10" t="s" s="7">
-        <v>29</v>
+        <v>10</v>
+      </c>
+      <c r="G10" s="10"/>
+      <c r="H10" t="s" s="9">
+        <v>32</v>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" t="s" s="3">
-        <v>30</v>
-      </c>
-      <c r="B11" t="s" s="7">
-        <v>28</v>
+        <v>33</v>
+      </c>
+      <c r="B11" t="s" s="9">
+        <v>31</v>
       </c>
       <c r="C11" s="4">
         <v>0</v>
@@ -2957,17 +3033,21 @@
       <c r="D11" s="5">
         <v>8192</v>
       </c>
-      <c r="E11" s="8"/>
+      <c r="E11" s="10"/>
       <c r="F11" t="s" s="7">
-        <v>31</v>
+        <v>10</v>
+      </c>
+      <c r="G11" s="10"/>
+      <c r="H11" t="s" s="9">
+        <v>34</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" t="s" s="3">
-        <v>32</v>
-      </c>
-      <c r="B12" t="s" s="7">
-        <v>28</v>
+        <v>35</v>
+      </c>
+      <c r="B12" t="s" s="9">
+        <v>31</v>
       </c>
       <c r="C12" s="4">
         <v>0</v>
@@ -2975,17 +3055,21 @@
       <c r="D12" s="5">
         <v>4096</v>
       </c>
-      <c r="E12" s="8"/>
+      <c r="E12" s="10"/>
       <c r="F12" t="s" s="7">
-        <v>33</v>
+        <v>10</v>
+      </c>
+      <c r="G12" s="10"/>
+      <c r="H12" t="s" s="9">
+        <v>36</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" t="s" s="3">
-        <v>34</v>
-      </c>
-      <c r="B13" t="s" s="7">
-        <v>28</v>
+        <v>37</v>
+      </c>
+      <c r="B13" t="s" s="9">
+        <v>31</v>
       </c>
       <c r="C13" s="4">
         <v>0</v>
@@ -2993,9 +3077,59 @@
       <c r="D13" s="5">
         <v>4096</v>
       </c>
-      <c r="E13" s="8"/>
+      <c r="E13" s="10"/>
       <c r="F13" t="s" s="7">
-        <v>35</v>
+        <v>10</v>
+      </c>
+      <c r="G13" t="b" s="6">
+        <v>1</v>
+      </c>
+      <c r="H13" t="s" s="9">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" t="s" s="3">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s" s="3">
+        <v>13</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5">
+        <v>8192</v>
+      </c>
+      <c r="E14" s="10"/>
+      <c r="F14" t="s" s="7">
+        <v>10</v>
+      </c>
+      <c r="G14" s="10"/>
+      <c r="H14" t="s" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" t="s" s="3">
+        <v>41</v>
+      </c>
+      <c r="B15" t="s" s="9">
+        <v>31</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5">
+        <v>16384</v>
+      </c>
+      <c r="E15" s="10"/>
+      <c r="F15" t="s" s="7">
+        <v>42</v>
+      </c>
+      <c r="G15" s="10"/>
+      <c r="H15" t="s" s="3">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>